<commit_message>
deploy: main → 990e3fdc1c14499b8ca89ab6aecbcf2ae9079fd0
</commit_message>
<xml_diff>
--- a/StructureDefinition-tk-endpoint.xlsx
+++ b/StructureDefinition-tk-endpoint.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AM$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AM$43</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1220" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="341">
   <si>
     <t>Property</t>
   </si>
@@ -538,77 +538,295 @@
 </t>
   </si>
   <si>
+    <t>Ändpunktsidentifierare, inklusive EHM:s motsvarande id</t>
+  </si>
+  <si>
+    <t>Identifier for the organization that is used to identify the endpoint across multiple disparate systems.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:system}
+</t>
+  </si>
+  <si>
+    <t>FiveWs.identifier</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier:ehmEndpointId</t>
+  </si>
+  <si>
+    <t>ehmEndpointId</t>
+  </si>
+  <si>
     <t>Identifies this endpoint across multiple systems</t>
   </si>
   <si>
-    <t>Identifier for the organization that is used to identify the endpoint across multiple disparate systems.</t>
-  </si>
-  <si>
-    <t>FiveWs.identifier</t>
-  </si>
-  <si>
-    <t>n/a</t>
-  </si>
-  <si>
-    <t>Endpoint.status</t>
-  </si>
-  <si>
-    <t>active | suspended | error | off | entered-in-error | test</t>
-  </si>
-  <si>
-    <t>The endpoint status represents the general expected availability of an endpoint.</t>
-  </si>
-  <si>
-    <t>This element is labeled as a modifier because the status contains codes that mark the endpoint as not currently valid. Temporary downtimes or other unexpected short-term changes in availability would not be represented in this property.</t>
-  </si>
-  <si>
-    <t>The status of the endpoint.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/endpoint-status|5.0.0</t>
-  </si>
-  <si>
-    <t>REQ-END-2</t>
-  </si>
-  <si>
-    <t>FiveWs.status</t>
-  </si>
-  <si>
-    <t>Endpoint.connectionType</t>
+    <t>REQ-WRT-4</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier:ehmEndpointId.id</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier.id</t>
+  </si>
+  <si>
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ele-1
+</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier:ehmEndpointId.extension</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier.extension</t>
+  </si>
+  <si>
+    <t>Additional content defined by implementations</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and managable, there is a strict set of governance applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier:ehmEndpointId.use</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier.use</t>
+  </si>
+  <si>
+    <t>usual | official | temp | secondary | old (If known)</t>
+  </si>
+  <si>
+    <t>The purpose of this identifier.</t>
+  </si>
+  <si>
+    <t>Applications can assume that an identifier is permanent unless it explicitly says that it is temporary.</t>
+  </si>
+  <si>
+    <t>Allows the appropriate identifier for a particular context of use to be selected from among a set of identifiers.</t>
+  </si>
+  <si>
+    <t>Identifies the purpose for this identifier, if known .</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/identifier-use|5.0.0</t>
+  </si>
+  <si>
+    <t>Identifier.use</t>
+  </si>
+  <si>
+    <t>Role.code or implied by context</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier:ehmEndpointId.type</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier.type</t>
   </si>
   <si>
     <t xml:space="preserve">CodeableConcept
 </t>
   </si>
   <si>
-    <t>Protokoll som ändpunkten stödjer</t>
-  </si>
-  <si>
-    <t>A coded value that represents the technical details of the usage of this endpoint, such as what WSDLs should be used in what way. (e.g. XDS.b/DICOM/cds-hook).</t>
-  </si>
-  <si>
-    <t>For additional connectivity details for the protocol, extensions will be used at this point, as in the XDS example. If there are multiple payload types or mimetypes they are all applicable for all connection types, and all have the same status.</t>
-  </si>
-  <si>
-    <t>example</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/endpoint-connection-type|5.0.0</t>
-  </si>
-  <si>
-    <t>REQ-END-8</t>
-  </si>
-  <si>
-    <t>FiveWs.class</t>
-  </si>
-  <si>
-    <t>Endpoint.name</t>
+    <t>Description of identifier</t>
+  </si>
+  <si>
+    <t>A coded type for the identifier that can be used to determine which identifier to use for a specific purpose.</t>
+  </si>
+  <si>
+    <t>This element deals only with general categories of identifiers.  It SHOULD not be used for codes that correspond 1..1 with the Identifier.system. Some identifiers may fall into multiple categories due to common usage.   Where the system is known, a type is unnecessary because the type is always part of the system definition. However systems often need to handle identifiers where the system is not known. There is not a 1:1 relationship between type and system, since many different systems have the same type.</t>
+  </si>
+  <si>
+    <t>Allows users to make use of identifiers when the identifier system is not known.</t>
+  </si>
+  <si>
+    <t>extensible</t>
+  </si>
+  <si>
+    <t>A coded type for an identifier that can be used to determine which identifier to use for a specific purpose.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/identifier-type|5.0.0</t>
+  </si>
+  <si>
+    <t>Identifier.type</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier:ehmEndpointId.system</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier.system</t>
+  </si>
+  <si>
+    <t>The namespace for the identifier value</t>
+  </si>
+  <si>
+    <t>Establishes the namespace for the value - that is, an absolute URL that describes a set values that are unique.</t>
+  </si>
+  <si>
+    <t>Identifier.system is always case sensitive.</t>
+  </si>
+  <si>
+    <t>There are many sets  of identifiers.  To perform matching of two identifiers, we need to know what set we're dealing with. The system identifies a particular set of unique identifiers.</t>
+  </si>
+  <si>
+    <t>http://electronichealth.se/fhir/NDI/Endpoint</t>
+  </si>
+  <si>
+    <t>http://www.acme.com/identifiers/patient</t>
+  </si>
+  <si>
+    <t>Identifier.system</t>
+  </si>
+  <si>
+    <t>II.root or Role.id.root</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier:ehmEndpointId.value</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier.value</t>
   </si>
   <si>
     <t xml:space="preserve">string
 </t>
   </si>
   <si>
+    <t>EHM:s logiska id (UUID) för samma ändpunkt i deras register</t>
+  </si>
+  <si>
+    <t>The portion of the identifier typically relevant to the user and which is unique within the context of the system.</t>
+  </si>
+  <si>
+    <t>If the value is a full URI, then the system SHALL be urn:ietf:rfc:3986.  The value's primary purpose is computational mapping.  As a result, it may be normalized for comparison purposes (e.g. removing non-significant whitespace, dashes, etc.)  A value formatted for human display can be conveyed using the [http://hl7.org/fhir/StructureDefinition/rendered-value](http://hl7.org/fhir/extensions/StructureDefinition-rendered-value.html)). Identifier.value is to be treated as case sensitive unless knowledge of the Identifier.system allows the processer to be confident that non-case-sensitive processing is safe.</t>
+  </si>
+  <si>
+    <t>123456</t>
+  </si>
+  <si>
+    <t>Identifier.value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ident-1
+</t>
+  </si>
+  <si>
+    <t>II.extension or II.root if system indicates OID or GUID (Or Role.id.extension or root)</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier:ehmEndpointId.period</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier.period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period
+</t>
+  </si>
+  <si>
+    <t>Time period when id is/was valid for use</t>
+  </si>
+  <si>
+    <t>Time period during which identifier is/was valid for use.</t>
+  </si>
+  <si>
+    <t>Identifier.period</t>
+  </si>
+  <si>
+    <t>Role.effectiveTime or implied by context</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier:ehmEndpointId.assigner</t>
+  </si>
+  <si>
+    <t>Endpoint.identifier.assigner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Organization|5.0.0)
+</t>
+  </si>
+  <si>
+    <t>Organization that issued id (may be just text)</t>
+  </si>
+  <si>
+    <t>Organization that issued/manages the identifier.</t>
+  </si>
+  <si>
+    <t>The Identifier.assigner may omit the .reference element and only contain a .display element reflecting the name or other textual information about the assigning organization.</t>
+  </si>
+  <si>
+    <t>Identifier.assigner</t>
+  </si>
+  <si>
+    <t>II.assigningAuthorityName but note that this is an improper use by the definition of the field.  Also Role.scoper</t>
+  </si>
+  <si>
+    <t>Endpoint.status</t>
+  </si>
+  <si>
+    <t>active | suspended | error | off | entered-in-error | test</t>
+  </si>
+  <si>
+    <t>The endpoint status represents the general expected availability of an endpoint.</t>
+  </si>
+  <si>
+    <t>This element is labeled as a modifier because the status contains codes that mark the endpoint as not currently valid. Temporary downtimes or other unexpected short-term changes in availability would not be represented in this property.</t>
+  </si>
+  <si>
+    <t>The status of the endpoint.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/endpoint-status|5.0.0</t>
+  </si>
+  <si>
+    <t>REQ-END-2</t>
+  </si>
+  <si>
+    <t>FiveWs.status</t>
+  </si>
+  <si>
+    <t>Endpoint.connectionType</t>
+  </si>
+  <si>
+    <t>Protokoll som ändpunkten stödjer</t>
+  </si>
+  <si>
+    <t>A coded value that represents the technical details of the usage of this endpoint, such as what WSDLs should be used in what way. (e.g. XDS.b/DICOM/cds-hook).</t>
+  </si>
+  <si>
+    <t>For additional connectivity details for the protocol, extensions will be used at this point, as in the XDS example. If there are multiple payload types or mimetypes they are all applicable for all connection types, and all have the same status.</t>
+  </si>
+  <si>
+    <t>example</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/endpoint-connection-type|5.0.0</t>
+  </si>
+  <si>
+    <t>REQ-END-8</t>
+  </si>
+  <si>
+    <t>FiveWs.class</t>
+  </si>
+  <si>
+    <t>Endpoint.name</t>
+  </si>
+  <si>
     <t>Ändpunktens namn</t>
   </si>
   <si>
@@ -637,9 +855,6 @@
   </si>
   <si>
     <t>The type of environment(s) exposed at this endpoint (dev, prod, test, etc.).</t>
-  </si>
-  <si>
-    <t>extensible</t>
   </si>
   <si>
     <t>http://hl7.org/fhir/ValueSet/endpoint-environment|5.0.0</t>
@@ -680,10 +895,6 @@
     <t>Endpoint.period</t>
   </si>
   <si>
-    <t xml:space="preserve">Period
-</t>
-  </si>
-  <si>
     <t>Interval the endpoint is expected to be operational</t>
   </si>
   <si>
@@ -702,32 +913,7 @@
     <t>Endpoint.period.id</t>
   </si>
   <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ele-1
-</t>
-  </si>
-  <si>
     <t>Endpoint.period.extension</t>
-  </si>
-  <si>
-    <t>Additional content defined by implementations</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and managable, there is a strict set of governance applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t>Extensions are always sliced by (at least) url</t>
-  </si>
-  <si>
-    <t>Element.extension</t>
   </si>
   <si>
     <t>Endpoint.period.start</t>
@@ -1227,7 +1413,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AM34"/>
+  <dimension ref="A1:AM43"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="36.30859375" customWidth="true" bestFit="true"/>
@@ -1249,12 +1435,12 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.53515625" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="32.7734375" customWidth="true" bestFit="true"/>
     <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
     <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="44.609375" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="84.33984375" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="47.29296875" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
@@ -1267,7 +1453,7 @@
     <col min="35" max="35" width="100.703125" customWidth="true"/>
     <col min="37" max="37" width="20.6171875" customWidth="true" bestFit="true"/>
     <col min="38" max="38" width="31.65234375" customWidth="true" bestFit="true"/>
-    <col min="39" max="39" width="21.4140625" customWidth="true" bestFit="true"/>
+    <col min="39" max="39" width="87.9765625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2623,7 +2809,7 @@
         <v>79</v>
       </c>
       <c r="H13" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I13" t="s" s="2">
         <v>77</v>
@@ -2677,16 +2863,14 @@
         <v>77</v>
       </c>
       <c r="AB13" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC13" t="s" s="2">
-        <v>77</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="AC13" s="2"/>
       <c r="AD13" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE13" t="s" s="2">
-        <v>77</v>
+        <v>139</v>
       </c>
       <c r="AF13" t="s" s="2">
         <v>161</v>
@@ -2707,26 +2891,28 @@
         <v>77</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AM13" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>167</v>
-      </c>
-      <c r="C14" s="2"/>
+        <v>161</v>
+      </c>
+      <c r="C14" t="s" s="2">
+        <v>169</v>
+      </c>
       <c r="D14" t="s" s="2">
         <v>77</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G14" t="s" s="2">
         <v>87</v>
@@ -2735,23 +2921,21 @@
         <v>88</v>
       </c>
       <c r="I14" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="J14" t="s" s="2">
         <v>88</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>108</v>
+        <v>162</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>169</v>
-      </c>
-      <c r="N14" t="s" s="2">
-        <v>170</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="N14" s="2"/>
       <c r="O14" s="2"/>
       <c r="P14" t="s" s="2">
         <v>77</v>
@@ -2776,13 +2960,13 @@
         <v>77</v>
       </c>
       <c r="X14" t="s" s="2">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="Y14" t="s" s="2">
-        <v>171</v>
+        <v>77</v>
       </c>
       <c r="Z14" t="s" s="2">
-        <v>172</v>
+        <v>77</v>
       </c>
       <c r="AA14" t="s" s="2">
         <v>77</v>
@@ -2800,13 +2984,13 @@
         <v>77</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="AG14" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AH14" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="AI14" t="s" s="2">
         <v>77</v>
@@ -2815,21 +2999,21 @@
         <v>100</v>
       </c>
       <c r="AK14" t="s" s="2">
+        <v>171</v>
+      </c>
+      <c r="AL14" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="AM14" t="s" s="2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="15" hidden="true">
+      <c r="A15" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="B15" t="s" s="2">
         <v>173</v>
-      </c>
-      <c r="AL14" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="AM14" t="s" s="2">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="2">
-        <v>175</v>
-      </c>
-      <c r="B15" t="s" s="2">
-        <v>175</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -2837,32 +3021,30 @@
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G15" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="G15" t="s" s="2">
-        <v>79</v>
-      </c>
       <c r="H15" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I15" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J15" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>176</v>
+        <v>89</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="N15" t="s" s="2">
-        <v>179</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="N15" s="2"/>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
         <v>77</v>
@@ -2887,11 +3069,13 @@
         <v>77</v>
       </c>
       <c r="X15" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="Y15" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="Y15" t="s" s="2">
+        <v>77</v>
+      </c>
       <c r="Z15" t="s" s="2">
-        <v>181</v>
+        <v>77</v>
       </c>
       <c r="AA15" t="s" s="2">
         <v>77</v>
@@ -2909,67 +3093,69 @@
         <v>77</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AG15" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH15" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="AH15" t="s" s="2">
-        <v>79</v>
-      </c>
       <c r="AI15" t="s" s="2">
-        <v>77</v>
+        <v>177</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="AK15" t="s" s="2">
-        <v>182</v>
+        <v>77</v>
       </c>
       <c r="AL15" t="s" s="2">
-        <v>183</v>
+        <v>77</v>
       </c>
       <c r="AM15" t="s" s="2">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
-        <v>77</v>
+        <v>155</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="H16" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I16" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J16" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>185</v>
+        <v>135</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>187</v>
-      </c>
-      <c r="N16" s="2"/>
+        <v>181</v>
+      </c>
+      <c r="N16" t="s" s="2">
+        <v>158</v>
+      </c>
       <c r="O16" s="2"/>
       <c r="P16" t="s" s="2">
         <v>77</v>
@@ -3006,48 +3192,48 @@
         <v>77</v>
       </c>
       <c r="AB16" t="s" s="2">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="AC16" t="s" s="2">
-        <v>77</v>
+        <v>182</v>
       </c>
       <c r="AD16" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE16" t="s" s="2">
-        <v>77</v>
+        <v>139</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH16" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="AI16" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ16" t="s" s="2">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>188</v>
+        <v>77</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>189</v>
+        <v>77</v>
       </c>
       <c r="AM16" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3064,22 +3250,26 @@
         <v>77</v>
       </c>
       <c r="I17" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="J17" t="s" s="2">
         <v>88</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>185</v>
+        <v>108</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>192</v>
-      </c>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
+        <v>187</v>
+      </c>
+      <c r="N17" t="s" s="2">
+        <v>188</v>
+      </c>
+      <c r="O17" t="s" s="2">
+        <v>189</v>
+      </c>
       <c r="P17" t="s" s="2">
         <v>77</v>
       </c>
@@ -3103,13 +3293,13 @@
         <v>77</v>
       </c>
       <c r="X17" t="s" s="2">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="Y17" t="s" s="2">
-        <v>77</v>
+        <v>190</v>
       </c>
       <c r="Z17" t="s" s="2">
-        <v>77</v>
+        <v>191</v>
       </c>
       <c r="AA17" t="s" s="2">
         <v>77</v>
@@ -3127,7 +3317,7 @@
         <v>77</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>78</v>
@@ -3148,15 +3338,15 @@
         <v>77</v>
       </c>
       <c r="AM17" t="s" s="2">
-        <v>166</v>
+        <v>193</v>
       </c>
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3167,7 +3357,7 @@
         <v>78</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H18" t="s" s="2">
         <v>77</v>
@@ -3179,16 +3369,20 @@
         <v>88</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>195</v>
-      </c>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
+        <v>198</v>
+      </c>
+      <c r="N18" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="O18" t="s" s="2">
+        <v>200</v>
+      </c>
       <c r="P18" t="s" s="2">
         <v>77</v>
       </c>
@@ -3212,11 +3406,13 @@
         <v>77</v>
       </c>
       <c r="X18" t="s" s="2">
-        <v>196</v>
-      </c>
-      <c r="Y18" s="2"/>
+        <v>201</v>
+      </c>
+      <c r="Y18" t="s" s="2">
+        <v>202</v>
+      </c>
       <c r="Z18" t="s" s="2">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="AA18" t="s" s="2">
         <v>77</v>
@@ -3234,13 +3430,13 @@
         <v>77</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH18" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI18" t="s" s="2">
         <v>77</v>
@@ -3255,15 +3451,15 @@
         <v>77</v>
       </c>
       <c r="AM18" t="s" s="2">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3277,7 +3473,7 @@
         <v>87</v>
       </c>
       <c r="H19" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I19" t="s" s="2">
         <v>77</v>
@@ -3286,18 +3482,20 @@
         <v>88</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>199</v>
+        <v>102</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>202</v>
-      </c>
-      <c r="O19" s="2"/>
+        <v>209</v>
+      </c>
+      <c r="O19" t="s" s="2">
+        <v>210</v>
+      </c>
       <c r="P19" t="s" s="2">
         <v>77</v>
       </c>
@@ -3306,10 +3504,10 @@
         <v>77</v>
       </c>
       <c r="S19" t="s" s="2">
-        <v>77</v>
+        <v>211</v>
       </c>
       <c r="T19" t="s" s="2">
-        <v>77</v>
+        <v>212</v>
       </c>
       <c r="U19" t="s" s="2">
         <v>77</v>
@@ -3345,7 +3543,7 @@
         <v>77</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>78</v>
@@ -3360,21 +3558,21 @@
         <v>100</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>203</v>
+        <v>77</v>
       </c>
       <c r="AL19" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AM19" t="s" s="2">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="20" hidden="true">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" t="s" s="2">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3382,30 +3580,32 @@
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H20" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I20" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>207</v>
-      </c>
-      <c r="N20" s="2"/>
+        <v>219</v>
+      </c>
+      <c r="N20" t="s" s="2">
+        <v>220</v>
+      </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>77</v>
@@ -3418,7 +3618,7 @@
         <v>77</v>
       </c>
       <c r="T20" t="s" s="2">
-        <v>77</v>
+        <v>221</v>
       </c>
       <c r="U20" t="s" s="2">
         <v>77</v>
@@ -3454,16 +3654,16 @@
         <v>77</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>204</v>
+        <v>222</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI20" t="s" s="2">
-        <v>77</v>
+        <v>223</v>
       </c>
       <c r="AJ20" t="s" s="2">
         <v>100</v>
@@ -3475,15 +3675,15 @@
         <v>77</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>208</v>
+        <v>226</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3497,7 +3697,7 @@
         <v>87</v>
       </c>
       <c r="H21" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I21" t="s" s="2">
         <v>77</v>
@@ -3506,17 +3706,15 @@
         <v>88</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>209</v>
+        <v>227</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>210</v>
+        <v>228</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>211</v>
-      </c>
-      <c r="N21" t="s" s="2">
-        <v>212</v>
-      </c>
+        <v>229</v>
+      </c>
+      <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>77</v>
@@ -3565,7 +3763,7 @@
         <v>77</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>208</v>
+        <v>230</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>78</v>
@@ -3580,21 +3778,21 @@
         <v>100</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>213</v>
+        <v>77</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>214</v>
+        <v>77</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>166</v>
+        <v>231</v>
       </c>
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>215</v>
+        <v>232</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>215</v>
+        <v>233</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3614,18 +3812,20 @@
         <v>77</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>89</v>
+        <v>234</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>216</v>
+        <v>235</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>217</v>
-      </c>
-      <c r="N22" s="2"/>
+        <v>236</v>
+      </c>
+      <c r="N22" t="s" s="2">
+        <v>237</v>
+      </c>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>77</v>
@@ -3674,7 +3874,7 @@
         <v>77</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>218</v>
+        <v>238</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>78</v>
@@ -3683,10 +3883,10 @@
         <v>87</v>
       </c>
       <c r="AI22" t="s" s="2">
-        <v>219</v>
+        <v>77</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="AK22" t="s" s="2">
         <v>77</v>
@@ -3695,47 +3895,47 @@
         <v>77</v>
       </c>
       <c r="AM22" t="s" s="2">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="23" hidden="true">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="23">
       <c r="A23" t="s" s="2">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>155</v>
+        <v>77</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I23" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>221</v>
+        <v>241</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>158</v>
+        <v>243</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -3761,60 +3961,60 @@
         <v>77</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>77</v>
+        <v>244</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>77</v>
+        <v>245</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AB23" t="s" s="2">
-        <v>138</v>
+        <v>77</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>223</v>
+        <v>77</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE23" t="s" s="2">
-        <v>139</v>
+        <v>77</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>224</v>
+        <v>240</v>
       </c>
       <c r="AG23" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>77</v>
+        <v>246</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>77</v>
+        <v>247</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>225</v>
+        <v>248</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>225</v>
+        <v>248</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3822,10 +4022,10 @@
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="G24" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="H24" t="s" s="2">
         <v>88</v>
@@ -3837,16 +4037,16 @@
         <v>88</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>226</v>
+        <v>196</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>227</v>
+        <v>249</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>228</v>
+        <v>250</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>229</v>
+        <v>251</v>
       </c>
       <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
@@ -3872,13 +4072,11 @@
         <v>77</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y24" t="s" s="2">
-        <v>77</v>
-      </c>
+        <v>252</v>
+      </c>
+      <c r="Y24" s="2"/>
       <c r="Z24" t="s" s="2">
-        <v>77</v>
+        <v>253</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>77</v>
@@ -3896,36 +4094,36 @@
         <v>77</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>230</v>
+        <v>248</v>
       </c>
       <c r="AG24" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AH24" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="AI24" t="s" s="2">
-        <v>231</v>
+        <v>77</v>
       </c>
       <c r="AJ24" t="s" s="2">
         <v>100</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>77</v>
+        <v>254</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>77</v>
+        <v>255</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>232</v>
+        <v>167</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>233</v>
+        <v>256</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>233</v>
+        <v>256</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3933,7 +4131,7 @@
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="G25" t="s" s="2">
         <v>87</v>
@@ -3948,24 +4146,20 @@
         <v>88</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>234</v>
+        <v>257</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>235</v>
-      </c>
-      <c r="N25" t="s" s="2">
-        <v>236</v>
-      </c>
+        <v>258</v>
+      </c>
+      <c r="N25" s="2"/>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="Q25" t="s" s="2">
-        <v>237</v>
-      </c>
+      <c r="Q25" s="2"/>
       <c r="R25" t="s" s="2">
         <v>77</v>
       </c>
@@ -4009,7 +4203,7 @@
         <v>77</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
@@ -4018,27 +4212,27 @@
         <v>87</v>
       </c>
       <c r="AI25" t="s" s="2">
-        <v>231</v>
+        <v>77</v>
       </c>
       <c r="AJ25" t="s" s="2">
         <v>100</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>77</v>
+        <v>259</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>77</v>
+        <v>260</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4049,29 +4243,27 @@
         <v>78</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J26" t="s" s="2">
         <v>88</v>
       </c>
-      <c r="I26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J26" t="s" s="2">
-        <v>77</v>
-      </c>
       <c r="K26" t="s" s="2">
-        <v>241</v>
+        <v>217</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>242</v>
+        <v>262</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>243</v>
-      </c>
-      <c r="N26" t="s" s="2">
-        <v>244</v>
-      </c>
+        <v>263</v>
+      </c>
+      <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
         <v>77</v>
@@ -4120,13 +4312,13 @@
         <v>77</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH26" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI26" t="s" s="2">
         <v>77</v>
@@ -4141,15 +4333,15 @@
         <v>77</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>77</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4160,7 +4352,7 @@
         <v>78</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>77</v>
@@ -4169,16 +4361,16 @@
         <v>77</v>
       </c>
       <c r="J27" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>216</v>
+        <v>265</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>217</v>
+        <v>266</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4205,13 +4397,11 @@
         <v>77</v>
       </c>
       <c r="X27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y27" t="s" s="2">
-        <v>77</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="Y27" s="2"/>
       <c r="Z27" t="s" s="2">
-        <v>77</v>
+        <v>267</v>
       </c>
       <c r="AA27" t="s" s="2">
         <v>77</v>
@@ -4229,19 +4419,19 @@
         <v>77</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>218</v>
+        <v>264</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="AI27" t="s" s="2">
-        <v>219</v>
+        <v>77</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>77</v>
@@ -4250,15 +4440,15 @@
         <v>77</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="28" hidden="true">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="28">
       <c r="A28" t="s" s="2">
-        <v>246</v>
+        <v>268</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>246</v>
+        <v>268</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4266,30 +4456,32 @@
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>135</v>
+        <v>269</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>136</v>
+        <v>270</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="N28" s="2"/>
+        <v>271</v>
+      </c>
+      <c r="N28" t="s" s="2">
+        <v>272</v>
+      </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>77</v>
@@ -4326,50 +4518,50 @@
         <v>77</v>
       </c>
       <c r="AB28" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="AC28" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="AC28" t="s" s="2">
+        <v>77</v>
+      </c>
       <c r="AD28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE28" t="s" s="2">
-        <v>139</v>
+        <v>77</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>224</v>
+        <v>268</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>77</v>
+        <v>273</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>247</v>
+        <v>274</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>246</v>
-      </c>
-      <c r="C29" t="s" s="2">
-        <v>248</v>
-      </c>
+        <v>274</v>
+      </c>
+      <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
         <v>77</v>
       </c>
@@ -4381,7 +4573,7 @@
         <v>79</v>
       </c>
       <c r="H29" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I29" t="s" s="2">
         <v>77</v>
@@ -4390,13 +4582,13 @@
         <v>77</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>249</v>
+        <v>275</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>251</v>
+        <v>277</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4447,7 +4639,7 @@
         <v>77</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>224</v>
+        <v>274</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
@@ -4459,60 +4651,58 @@
         <v>77</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>252</v>
+        <v>77</v>
       </c>
       <c r="AL29" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="30" hidden="true">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="30">
       <c r="A30" t="s" s="2">
-        <v>253</v>
+        <v>278</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>253</v>
+        <v>278</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>254</v>
+        <v>77</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H30" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I30" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="J30" t="s" s="2">
         <v>88</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>135</v>
+        <v>227</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>256</v>
+        <v>280</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="O30" t="s" s="2">
-        <v>159</v>
-      </c>
+        <v>281</v>
+      </c>
+      <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>77</v>
       </c>
@@ -4560,36 +4750,36 @@
         <v>77</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>257</v>
+        <v>278</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>77</v>
+        <v>282</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>77</v>
+        <v>283</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>258</v>
+        <v>284</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>258</v>
+        <v>284</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4597,32 +4787,30 @@
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G31" t="s" s="2">
         <v>87</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>176</v>
+        <v>89</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>259</v>
+        <v>174</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>261</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="N31" s="2"/>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>77</v>
@@ -4647,11 +4835,13 @@
         <v>77</v>
       </c>
       <c r="X31" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="Y31" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="Y31" t="s" s="2">
+        <v>77</v>
+      </c>
       <c r="Z31" t="s" s="2">
-        <v>262</v>
+        <v>77</v>
       </c>
       <c r="AA31" t="s" s="2">
         <v>77</v>
@@ -4669,40 +4859,40 @@
         <v>77</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>258</v>
+        <v>176</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI31" t="s" s="2">
-        <v>77</v>
+        <v>177</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>263</v>
+        <v>77</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>264</v>
+        <v>285</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>264</v>
+        <v>285</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>77</v>
+        <v>155</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
@@ -4718,19 +4908,19 @@
         <v>77</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>265</v>
+        <v>180</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>266</v>
+        <v>181</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>267</v>
+        <v>158</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -4756,31 +4946,31 @@
         <v>77</v>
       </c>
       <c r="X32" t="s" s="2">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="Y32" t="s" s="2">
-        <v>268</v>
+        <v>77</v>
       </c>
       <c r="Z32" t="s" s="2">
-        <v>269</v>
+        <v>77</v>
       </c>
       <c r="AA32" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AB32" t="s" s="2">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="AC32" t="s" s="2">
-        <v>77</v>
+        <v>182</v>
       </c>
       <c r="AD32" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE32" t="s" s="2">
-        <v>77</v>
+        <v>139</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>264</v>
+        <v>183</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
@@ -4792,7 +4982,7 @@
         <v>77</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>77</v>
@@ -4801,15 +4991,15 @@
         <v>77</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>270</v>
+        <v>286</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>270</v>
+        <v>286</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -4817,7 +5007,7 @@
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G33" t="s" s="2">
         <v>87</v>
@@ -4832,16 +5022,16 @@
         <v>88</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>271</v>
+        <v>287</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>272</v>
+        <v>288</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>273</v>
+        <v>289</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>274</v>
+        <v>290</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -4891,36 +5081,36 @@
         <v>77</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>270</v>
+        <v>291</v>
       </c>
       <c r="AG33" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AH33" t="s" s="2">
         <v>87</v>
       </c>
       <c r="AI33" t="s" s="2">
-        <v>77</v>
+        <v>292</v>
       </c>
       <c r="AJ33" t="s" s="2">
         <v>100</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>275</v>
+        <v>77</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="34" hidden="true">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="34">
       <c r="A34" t="s" s="2">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4931,34 +5121,36 @@
         <v>78</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H34" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I34" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>185</v>
+        <v>287</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>277</v>
+        <v>295</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>279</v>
+        <v>297</v>
       </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="Q34" s="2"/>
+      <c r="Q34" t="s" s="2">
+        <v>298</v>
+      </c>
       <c r="R34" t="s" s="2">
         <v>77</v>
       </c>
@@ -5002,16 +5194,16 @@
         <v>77</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>276</v>
+        <v>299</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI34" t="s" s="2">
-        <v>77</v>
+        <v>292</v>
       </c>
       <c r="AJ34" t="s" s="2">
         <v>100</v>
@@ -5023,11 +5215,1004 @@
         <v>77</v>
       </c>
       <c r="AM34" t="s" s="2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="B35" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="C35" s="2"/>
+      <c r="D35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E35" s="2"/>
+      <c r="F35" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G35" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H35" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="I35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K35" t="s" s="2">
+        <v>302</v>
+      </c>
+      <c r="L35" t="s" s="2">
+        <v>303</v>
+      </c>
+      <c r="M35" t="s" s="2">
+        <v>304</v>
+      </c>
+      <c r="N35" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="O35" s="2"/>
+      <c r="P35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q35" s="2"/>
+      <c r="R35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF35" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="AG35" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH35" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ35" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM35" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" hidden="true">
+      <c r="A36" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="B36" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E36" s="2"/>
+      <c r="F36" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G36" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K36" t="s" s="2">
+        <v>217</v>
+      </c>
+      <c r="L36" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="M36" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q36" s="2"/>
+      <c r="R36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF36" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="AG36" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH36" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI36" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AJ36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AK36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM36" t="s" s="2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="37" hidden="true">
+      <c r="A37" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="B37" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E37" s="2"/>
+      <c r="F37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G37" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K37" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L37" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="M37" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="P37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q37" s="2"/>
+      <c r="R37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB37" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AC37" s="2"/>
+      <c r="AD37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE37" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="AF37" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="AG37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH37" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ37" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="AK37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM37" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="B38" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="C38" t="s" s="2">
+        <v>309</v>
+      </c>
+      <c r="D38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E38" s="2"/>
+      <c r="F38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G38" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H38" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="I38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K38" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="L38" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="M38" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="N38" s="2"/>
+      <c r="O38" s="2"/>
+      <c r="P38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q38" s="2"/>
+      <c r="R38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF38" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="AG38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH38" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ38" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="AK38" t="s" s="2">
+        <v>313</v>
+      </c>
+      <c r="AL38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM38" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" hidden="true">
+      <c r="A39" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="B39" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="E39" s="2"/>
+      <c r="F39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G39" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I39" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="J39" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K39" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L39" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="M39" t="s" s="2">
+        <v>317</v>
+      </c>
+      <c r="N39" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="O39" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="P39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q39" s="2"/>
+      <c r="R39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF39" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="AG39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH39" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ39" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="AK39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM39" t="s" s="2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="B40" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E40" s="2"/>
+      <c r="F40" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="G40" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H40" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="I40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J40" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K40" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="L40" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="M40" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="N40" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="O40" s="2"/>
+      <c r="P40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q40" s="2"/>
+      <c r="R40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X40" t="s" s="2">
+        <v>252</v>
+      </c>
+      <c r="Y40" s="2"/>
+      <c r="Z40" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="AA40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF40" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="AG40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH40" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ40" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK40" t="s" s="2">
+        <v>324</v>
+      </c>
+      <c r="AL40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM40" t="s" s="2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="41" hidden="true">
+      <c r="A41" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="B41" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E41" s="2"/>
+      <c r="F41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G41" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J41" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K41" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="L41" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="M41" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="N41" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="O41" s="2"/>
+      <c r="P41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q41" s="2"/>
+      <c r="R41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X41" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="Y41" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="Z41" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="AA41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF41" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AG41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH41" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ41" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL41" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM41" t="s" s="2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="2">
+        <v>331</v>
+      </c>
+      <c r="B42" t="s" s="2">
+        <v>331</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E42" s="2"/>
+      <c r="F42" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="G42" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H42" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="I42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J42" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K42" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="L42" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="M42" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="N42" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="O42" s="2"/>
+      <c r="P42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q42" s="2"/>
+      <c r="R42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF42" t="s" s="2">
+        <v>331</v>
+      </c>
+      <c r="AG42" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AH42" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ42" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK42" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="AL42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM42" t="s" s="2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="43" hidden="true">
+      <c r="A43" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="B43" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K43" t="s" s="2">
+        <v>217</v>
+      </c>
+      <c r="L43" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="M43" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="O43" s="2"/>
+      <c r="P43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q43" s="2"/>
+      <c r="R43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF43" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="AG43" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ43" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM43" t="s" s="2">
         <v>77</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM34">
+  <autoFilter ref="A1:AM43">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -5037,7 +6222,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI33">
+  <conditionalFormatting sqref="A2:AI42">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>